<commit_message>
Atualiza Tabela Mestre: sincronizacao de novos inscritos e confirmacao de aviso WhatsApp (Jose Carlos e Angelica)
</commit_message>
<xml_diff>
--- a/coleta/PILOTO OFICIAL/00_CADASTRO_TRIAGEM_E_TCLE/TABELA_MESTRE_IDENTIFICACAO_PARTICIPANTES.xlsx
+++ b/coleta/PILOTO OFICIAL/00_CADASTRO_TRIAGEM_E_TCLE/TABELA_MESTRE_IDENTIFICACAO_PARTICIPANTES.xlsx
@@ -4982,7 +4982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5358,7 +5358,7 @@
       <c r="R4" s="38" t="inlineStr"/>
       <c r="S4" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       <c r="R5" s="38" t="inlineStr"/>
       <c r="S5" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Apenas sustentar na parada de mãos (&gt;= 3s) | Nota: Aluno do pesquisador (Guilherme): sustenta 3s livre com segurança; HSW ainda em desenvolvimento. | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Apenas sustentar na parada de mãos (&gt;= 3s) | Nota: Aluno do pesquisador (Guilherme): sustenta 3s livre com segurança; HSW ainda em desenvolvimento.</t>
         </is>
       </c>
     </row>
@@ -5496,7 +5496,7 @@
       <c r="R6" s="38" t="inlineStr"/>
       <c r="S6" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições</t>
         </is>
       </c>
     </row>
@@ -5565,7 +5565,7 @@
       <c r="R7" s="38" t="inlineStr"/>
       <c r="S7" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5634,7 @@
       <c r="R8" s="38" t="inlineStr"/>
       <c r="S8" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Apenas sustentar na parada de mãos | Obs Lesão: Subluxacao posterior do ombro direito, gerando muita instabilidade! Atualmente não tenho dor e esta com mais estabilidade. Já estou treinando normal! | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Apenas sustentar na parada de mãos | Obs Lesão: Subluxacao posterior do ombro direito, gerando muita instabilidade! Atualmente não tenho dor e esta com mais estabilidade. Já estou treinando normal!</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       <c r="S9" s="37" t="inlineStr">
         <is>
           <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Obs Lesão: Fui virar um mortal e quando lancei as mãos pro alto senti uma dor no ombro direito, essa dor vem diminuindo desde então mas em alguns movimentos percebo que ela ainda está aqui. Parado ou andando isso não atrapalha no meu handstand. 
-Obs. Não fui ao médico. | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+Obs. Não fui ao médico.</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5773,7 @@
       <c r="R10" s="38" t="inlineStr"/>
       <c r="S10" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5842,7 @@
       <c r="R11" s="38" t="inlineStr"/>
       <c r="S11" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Obs Lesão: Lesão no punho, derrame articular em fevereiro. Atualmente, sem dores para paradas de mãos. | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Obs Lesão: Lesão no punho, derrame articular em fevereiro. Atualmente, sem dores para paradas de mãos.</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,145 @@
       <c r="R12" s="38" t="inlineStr"/>
       <c r="S12" s="37" t="inlineStr">
         <is>
-          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 22/09/2026 (Previsão de início em Outubro).</t>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>22/09/2026 10:56:34</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>José Carlos Targas</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>José Targas</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>20/05/1985 (41 anos)</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>16991647323</t>
+        </is>
+      </c>
+      <c r="G13" s="38" t="inlineStr"/>
+      <c r="H13" s="37" t="inlineStr">
+        <is>
+          <t>josecarlostargas@gmail.com</t>
+        </is>
+      </c>
+      <c r="I13" s="37" t="inlineStr"/>
+      <c r="J13" s="38" t="inlineStr"/>
+      <c r="K13" s="38" t="inlineStr"/>
+      <c r="L13" s="37" t="inlineStr">
+        <is>
+          <t>Sexta-feira, Sábado</t>
+        </is>
+      </c>
+      <c r="M13" s="37" t="inlineStr">
+        <is>
+          <t>10h as 12h, 18h as 20h</t>
+        </is>
+      </c>
+      <c r="N13" s="37" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="O13" s="41" t="inlineStr">
+        <is>
+          <t>Avisado / Aguardando Início (Outubro)</t>
+        </is>
+      </c>
+      <c r="P13" s="38" t="inlineStr"/>
+      <c r="Q13" s="38" t="inlineStr"/>
+      <c r="R13" s="38" t="inlineStr"/>
+      <c r="S13" s="37" t="inlineStr">
+        <is>
+          <t>Triado via Formulários Oficiais. | Critério HS: Ambas condições | Avisado via WhatsApp em 23/09/2026 (Previsão de início em Outubro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>22/09/2026 21:08:29</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Angélica Oliveira Leonel Silva</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Angélica Silva</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>09/07/1993 (33 anos)</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>16982152303</t>
+        </is>
+      </c>
+      <c r="G14" s="38" t="inlineStr"/>
+      <c r="H14" s="37" t="inlineStr">
+        <is>
+          <t>angelica.leonel7@hotmail.com</t>
+        </is>
+      </c>
+      <c r="I14" s="37" t="inlineStr"/>
+      <c r="J14" s="38" t="inlineStr"/>
+      <c r="K14" s="38" t="inlineStr"/>
+      <c r="L14" s="37" t="inlineStr">
+        <is>
+          <t>Sexta-feira, Sábado</t>
+        </is>
+      </c>
+      <c r="M14" s="37" t="inlineStr">
+        <is>
+          <t>8h as 10h, 18h as 20h</t>
+        </is>
+      </c>
+      <c r="N14" s="37" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="O14" s="41" t="inlineStr">
+        <is>
+          <t>Avisado / Aguardando Início (Outubro)</t>
+        </is>
+      </c>
+      <c r="P14" s="38" t="inlineStr"/>
+      <c r="Q14" s="38" t="inlineStr"/>
+      <c r="R14" s="38" t="inlineStr"/>
+      <c r="S14" s="37" t="inlineStr">
+        <is>
+          <t>Triado via Formulários Oficiais. | Critério HS: Apenas sustentar na parada de mãos | Obs Lesão: Tendinite e bursite no ombro esquerdo | Avisado via WhatsApp em 23/09/2026 (Previsão de início em Outubro).</t>
         </is>
       </c>
     </row>

</xml_diff>